<commit_message>
Correcion nombres a borrar
</commit_message>
<xml_diff>
--- a/VALORIZADO FALTANTES IMPO.xlsx
+++ b/VALORIZADO FALTANTES IMPO.xlsx
@@ -391,13 +391,13 @@
     <t>Valorizado</t>
   </si>
   <si>
-    <t>Período: 31/10/2025 09:44:16</t>
+    <t>Período: 31/10/2025 12:37:31</t>
   </si>
   <si>
     <t>COLGAAP</t>
   </si>
   <si>
-    <t>Fecha y hora de generación: 23/10/2025 09:52:47</t>
+    <t>Fecha y hora de generación: 27/10/2025 12:37:55</t>
   </si>
 </sst>
 </file>
@@ -1736,13 +1736,13 @@
         <v>119</v>
       </c>
       <c r="J35">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="K35">
         <v>18048.24</v>
       </c>
       <c r="L35">
-        <v>14185916.64</v>
+        <v>14294206.08</v>
       </c>
     </row>
     <row r="36" spans="1:12">

</xml_diff>

<commit_message>
prueba ale tiene muchas diferencias en el archivo generado por el validador
</commit_message>
<xml_diff>
--- a/VALORIZADO FALTANTES IMPO.xlsx
+++ b/VALORIZADO FALTANTES IMPO.xlsx
@@ -1,39 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jlopez\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{398EA981-CB44-4DBE-8D08-18C4ED10B4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Valorizado" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="130">
   <si>
     <t>Categoría</t>
   </si>
@@ -77,6 +58,18 @@
     <t>Categoría producto</t>
   </si>
   <si>
+    <t>7059</t>
+  </si>
+  <si>
+    <t>7086</t>
+  </si>
+  <si>
+    <t>235383</t>
+  </si>
+  <si>
+    <t>994349</t>
+  </si>
+  <si>
     <t>1824680C1</t>
   </si>
   <si>
@@ -119,6 +112,12 @@
     <t>X8870342</t>
   </si>
   <si>
+    <t>4302312</t>
+  </si>
+  <si>
+    <t>4304615</t>
+  </si>
+  <si>
     <t>128462/128947ARM</t>
   </si>
   <si>
@@ -143,6 +142,9 @@
     <t>R802689/R802447</t>
   </si>
   <si>
+    <t>4302670</t>
+  </si>
+  <si>
     <t>ES423L ELG/THK</t>
   </si>
   <si>
@@ -161,7 +163,10 @@
     <t>5556503/3MM</t>
   </si>
   <si>
-    <t>4303796/4301527WAP</t>
+    <t>14897</t>
+  </si>
+  <si>
+    <t>17515</t>
   </si>
   <si>
     <t>126180WAP</t>
@@ -350,9 +355,6 @@
     <t>CORREA PARA COLUMBIA SERIE60 12LT</t>
   </si>
   <si>
-    <t>PIÑON DE 4TA EJE CORREDIZO 4205</t>
-  </si>
-  <si>
     <t>ARANDELA SATELITE DIVISOR 46 LBS PLANA</t>
   </si>
   <si>
@@ -374,9 +376,6 @@
     <t>USA</t>
   </si>
   <si>
-    <t>WAP/TRANSMISION</t>
-  </si>
-  <si>
     <t>WAP/DIFERENCIAL-CARDAN</t>
   </si>
   <si>
@@ -398,20 +397,20 @@
     <t>Valorizado</t>
   </si>
   <si>
-    <t>Período: 30/11/2025 12:29:18</t>
+    <t>Período: 29/11/2025 22:19:30</t>
   </si>
   <si>
     <t>COLGAAP</t>
   </si>
   <si>
-    <t>Fecha y hora de generación: 01/11/2025 12:29:51</t>
+    <t>Fecha y hora de generación: 04/11/2025 22:20:04</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,16 +503,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -521,31 +514,28 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -583,7 +573,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -617,7 +607,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -652,10 +641,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -828,130 +816,130 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L51"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="I7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-    </row>
-    <row r="5" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I7" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="7">
-        <v>7059</v>
-      </c>
-      <c r="C10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" t="s">
-        <v>111</v>
-      </c>
       <c r="F10" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="I10" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -963,27 +951,27 @@
         <v>111634.66</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7">
-        <v>7086</v>
+      <c r="B11" t="s">
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="I11" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -995,27 +983,27 @@
         <v>140713.63</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="7">
-        <v>235383</v>
+      <c r="B12" t="s">
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I12" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -1027,27 +1015,27 @@
         <v>55096.74</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="7">
-        <v>994349</v>
+      <c r="B13" t="s">
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="I13" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -1059,27 +1047,27 @@
         <v>574141.24</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F14" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I14" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J14">
         <v>2</v>
@@ -1091,59 +1079,59 @@
         <v>41733.82</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="E15" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="I15" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J15">
         <v>5</v>
       </c>
       <c r="K15">
-        <v>69586.600000000006</v>
+        <v>69586.60000000001</v>
       </c>
       <c r="L15">
         <v>347933</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I16" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1155,27 +1143,27 @@
         <v>354697.76</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="I17" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J17">
         <v>7</v>
@@ -1187,59 +1175,59 @@
         <v>492522.59</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12">
       <c r="A18" t="s">
         <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F18" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J18">
         <v>12</v>
       </c>
       <c r="K18">
-        <v>525495.80000000005</v>
+        <v>525495.8</v>
       </c>
       <c r="L18">
-        <v>6305949.5999999996</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+        <v>6305949.6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" t="s">
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I19" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J19">
         <v>4</v>
@@ -1251,59 +1239,59 @@
         <v>209726.48</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12">
       <c r="A20" t="s">
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D20" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E20" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F20" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="I20" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J20">
         <v>1</v>
       </c>
       <c r="K20">
-        <v>558922.19999999995</v>
+        <v>558922.2</v>
       </c>
       <c r="L20">
-        <v>558922.19999999995</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+        <v>558922.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21" t="s">
         <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="E21" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I21" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J21">
         <v>2</v>
@@ -1315,27 +1303,27 @@
         <v>219780.82</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12">
       <c r="A22" t="s">
         <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="I22" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1347,59 +1335,59 @@
         <v>237833.89</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12">
       <c r="A23" t="s">
         <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I23" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J23">
         <v>20</v>
       </c>
       <c r="K23">
-        <v>297747.46999999997</v>
+        <v>297747.47</v>
       </c>
       <c r="L23">
-        <v>5954949.4000000004</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+        <v>5954949.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" t="s">
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E24" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I24" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J24">
         <v>2</v>
@@ -1411,91 +1399,91 @@
         <v>189696.46</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12">
       <c r="A25" t="s">
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E25" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="I25" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J25">
         <v>1</v>
       </c>
       <c r="K25">
-        <v>150117.48000000001</v>
+        <v>150117.48</v>
       </c>
       <c r="L25">
-        <v>150117.48000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+        <v>150117.48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" t="s">
         <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F26" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="I26" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J26">
         <v>1</v>
       </c>
       <c r="K26">
-        <v>25537.919999999998</v>
+        <v>25537.92</v>
       </c>
       <c r="L26">
-        <v>25537.919999999998</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+        <v>25537.92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" t="s">
         <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D27" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F27" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I27" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J27">
         <v>5</v>
@@ -1507,59 +1495,59 @@
         <v>18205.05</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12">
       <c r="A28" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="7">
-        <v>4302312</v>
+      <c r="B28" t="s">
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D28" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F28" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I28" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28">
-        <v>20800.669999999998</v>
+        <v>20800.67</v>
       </c>
       <c r="L28">
-        <v>41601.339999999997</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+        <v>41601.34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" t="s">
         <v>12</v>
       </c>
-      <c r="B29" s="7">
-        <v>4304615</v>
+      <c r="B29" t="s">
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D29" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E29" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F29" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I29" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J29">
         <v>47</v>
@@ -1571,59 +1559,59 @@
         <v>185027.25</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12">
       <c r="A30" t="s">
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="E30" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F30" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="I30" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J30">
         <v>3</v>
       </c>
       <c r="K30">
-        <v>312918.09000000003</v>
+        <v>312918.09</v>
       </c>
       <c r="L30">
         <v>938754.27</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12">
       <c r="A31" t="s">
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D31" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="E31" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F31" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I31" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J31">
         <v>1</v>
@@ -1635,27 +1623,27 @@
         <v>206249.01</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12">
       <c r="A32" t="s">
         <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D32" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F32" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I32" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -1667,27 +1655,27 @@
         <v>2444357.96</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12">
       <c r="A33" t="s">
         <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E33" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="F33" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I33" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -1699,27 +1687,27 @@
         <v>216538.69</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12">
       <c r="A34" t="s">
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D34" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E34" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F34" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="I34" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -1731,91 +1719,91 @@
         <v>286676.26</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12">
       <c r="A35" t="s">
         <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E35" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="F35" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I35" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J35">
         <v>792</v>
       </c>
       <c r="K35">
-        <v>18048.240000000002</v>
+        <v>18048.24</v>
       </c>
       <c r="L35">
         <v>14294206.08</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12">
       <c r="A36" t="s">
         <v>12</v>
       </c>
       <c r="B36" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D36" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="E36" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F36" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I36" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J36">
         <v>60</v>
       </c>
       <c r="K36">
-        <v>20614.169999999998</v>
+        <v>20614.17</v>
       </c>
       <c r="L36">
         <v>1236850.2</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12">
       <c r="A37" t="s">
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D37" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E37" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F37" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I37" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J37">
         <v>13</v>
@@ -1824,30 +1812,30 @@
         <v>162426.15</v>
       </c>
       <c r="L37">
-        <v>2111539.9500000002</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+        <v>2111539.95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
       <c r="A38" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="7">
-        <v>4302670</v>
+      <c r="B38" t="s">
+        <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D38" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F38" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I38" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J38">
         <v>1</v>
@@ -1859,27 +1847,27 @@
         <v>261801.89</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12">
       <c r="A39" t="s">
         <v>12</v>
       </c>
       <c r="B39" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="E39" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F39" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="I39" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J39">
         <v>1</v>
@@ -1891,27 +1879,27 @@
         <v>75557.81</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12">
       <c r="A40" t="s">
         <v>12</v>
       </c>
       <c r="B40" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C40" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D40" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E40" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F40" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I40" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J40">
         <v>19</v>
@@ -1920,30 +1908,30 @@
         <v>122009.29</v>
       </c>
       <c r="L40">
-        <v>2318176.5099999998</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+        <v>2318176.51</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
       <c r="A41" t="s">
         <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C41" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D41" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E41" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F41" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I41" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -1955,27 +1943,27 @@
         <v>114045.11</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12">
       <c r="A42" t="s">
         <v>12</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="E42" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F42" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I42" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J42">
         <v>360</v>
@@ -1984,30 +1972,30 @@
         <v>3512.14</v>
       </c>
       <c r="L42">
-        <v>1264370.3999999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+        <v>1264370.4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
       <c r="A43" t="s">
         <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C43" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D43" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E43" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F43" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="I43" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J43">
         <v>364</v>
@@ -2019,27 +2007,27 @@
         <v>4607894.2</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12">
       <c r="A44" t="s">
         <v>12</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D44" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E44" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F44" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I44" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J44">
         <v>8</v>
@@ -2051,27 +2039,27 @@
         <v>1838804.96</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12">
       <c r="A45" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="7">
-        <v>14897</v>
+      <c r="B45" t="s">
+        <v>49</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D45" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="E45" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F45" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I45" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J45">
         <v>60</v>
@@ -2083,27 +2071,27 @@
         <v>39833.4</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12">
       <c r="A46" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="7">
-        <v>17515</v>
+      <c r="B46" t="s">
+        <v>50</v>
       </c>
       <c r="C46" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D46" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E46" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F46" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="I46" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J46">
         <v>1</v>
@@ -2115,195 +2103,163 @@
         <v>12173.17</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12">
       <c r="A47" t="s">
         <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C47" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="D47" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E47" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F47" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="I47" t="s">
+        <v>121</v>
+      </c>
+      <c r="J47">
+        <v>4</v>
+      </c>
+      <c r="K47">
+        <v>9156.48</v>
+      </c>
+      <c r="L47">
+        <v>36625.92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
+      <c r="A48" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" t="s">
+        <v>52</v>
+      </c>
+      <c r="C48" t="s">
+        <v>73</v>
+      </c>
+      <c r="D48" t="s">
+        <v>114</v>
+      </c>
+      <c r="E48" t="s">
+        <v>73</v>
+      </c>
+      <c r="F48" t="s">
+        <v>73</v>
+      </c>
+      <c r="I48" t="s">
+        <v>121</v>
+      </c>
+      <c r="J48">
+        <v>1</v>
+      </c>
+      <c r="K48">
+        <v>15384.67</v>
+      </c>
+      <c r="L48">
+        <v>15384.67</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
+      <c r="A49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" t="s">
+        <v>74</v>
+      </c>
+      <c r="D49" t="s">
         <v>115</v>
       </c>
-      <c r="J47">
+      <c r="E49" t="s">
+        <v>74</v>
+      </c>
+      <c r="F49" t="s">
+        <v>74</v>
+      </c>
+      <c r="I49" t="s">
+        <v>121</v>
+      </c>
+      <c r="J49">
+        <v>2</v>
+      </c>
+      <c r="K49">
+        <v>193066.84</v>
+      </c>
+      <c r="L49">
+        <v>386133.68</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
+      <c r="A50" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" t="s">
+        <v>74</v>
+      </c>
+      <c r="D50" t="s">
+        <v>116</v>
+      </c>
+      <c r="E50" t="s">
+        <v>74</v>
+      </c>
+      <c r="F50" t="s">
+        <v>74</v>
+      </c>
+      <c r="I50" t="s">
+        <v>121</v>
+      </c>
+      <c r="J50">
+        <v>5</v>
+      </c>
+      <c r="K50">
+        <v>26517.61</v>
+      </c>
+      <c r="L50">
+        <v>132588.05</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
+      <c r="A51" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" t="s">
+        <v>75</v>
+      </c>
+      <c r="D51" t="s">
+        <v>117</v>
+      </c>
+      <c r="E51" t="s">
+        <v>119</v>
+      </c>
+      <c r="F51" t="s">
+        <v>119</v>
+      </c>
+      <c r="I51" t="s">
+        <v>121</v>
+      </c>
+      <c r="J51">
         <v>1</v>
       </c>
-      <c r="K47">
-        <v>163002.70000000001</v>
-      </c>
-      <c r="L47">
-        <v>163002.70000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" t="s">
-        <v>106</v>
-      </c>
-      <c r="E48" t="s">
-        <v>64</v>
-      </c>
-      <c r="F48" t="s">
-        <v>114</v>
-      </c>
-      <c r="I48" t="s">
-        <v>115</v>
-      </c>
-      <c r="J48">
-        <v>4</v>
-      </c>
-      <c r="K48">
-        <v>9156.48</v>
-      </c>
-      <c r="L48">
-        <v>36625.919999999998</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" t="s">
-        <v>44</v>
-      </c>
-      <c r="C49" t="s">
-        <v>65</v>
-      </c>
-      <c r="D49" t="s">
-        <v>107</v>
-      </c>
-      <c r="E49" t="s">
-        <v>65</v>
-      </c>
-      <c r="F49" t="s">
-        <v>65</v>
-      </c>
-      <c r="I49" t="s">
-        <v>115</v>
-      </c>
-      <c r="J49">
-        <v>1</v>
-      </c>
-      <c r="K49">
-        <v>15384.67</v>
-      </c>
-      <c r="L49">
-        <v>15384.67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>12</v>
-      </c>
-      <c r="B50" t="s">
-        <v>45</v>
-      </c>
-      <c r="C50" t="s">
-        <v>66</v>
-      </c>
-      <c r="D50" t="s">
-        <v>108</v>
-      </c>
-      <c r="E50" t="s">
-        <v>66</v>
-      </c>
-      <c r="F50" t="s">
-        <v>66</v>
-      </c>
-      <c r="I50" t="s">
-        <v>115</v>
-      </c>
-      <c r="J50">
-        <v>2</v>
-      </c>
-      <c r="K50">
-        <v>193066.84</v>
-      </c>
-      <c r="L50">
-        <v>386133.68</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>12</v>
-      </c>
-      <c r="B51" t="s">
-        <v>46</v>
-      </c>
-      <c r="C51" t="s">
-        <v>66</v>
-      </c>
-      <c r="D51" t="s">
-        <v>109</v>
-      </c>
-      <c r="E51" t="s">
-        <v>66</v>
-      </c>
-      <c r="F51" t="s">
-        <v>66</v>
-      </c>
-      <c r="I51" t="s">
-        <v>115</v>
-      </c>
-      <c r="J51">
-        <v>5</v>
-      </c>
       <c r="K51">
-        <v>26517.61</v>
+        <v>39099.54</v>
       </c>
       <c r="L51">
-        <v>132588.04999999999</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>12</v>
-      </c>
-      <c r="B52" t="s">
-        <v>47</v>
-      </c>
-      <c r="C52" t="s">
-        <v>67</v>
-      </c>
-      <c r="D52" t="s">
-        <v>110</v>
-      </c>
-      <c r="E52" t="s">
-        <v>112</v>
-      </c>
-      <c r="F52" t="s">
-        <v>112</v>
-      </c>
-      <c r="I52" t="s">
-        <v>115</v>
-      </c>
-      <c r="J52">
-        <v>1</v>
-      </c>
-      <c r="K52">
-        <v>39099.54</v>
-      </c>
-      <c r="L52">
         <v>39099.54</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar inv general automatico
</commit_message>
<xml_diff>
--- a/VALORIZADO FALTANTES IMPO.xlsx
+++ b/VALORIZADO FALTANTES IMPO.xlsx
@@ -400,13 +400,13 @@
     <t>Valorizado</t>
   </si>
   <si>
-    <t>Período: 30/11/2025 08:47:22</t>
+    <t>Período: 31/12/2025 08:45:38</t>
   </si>
   <si>
     <t>COLGAAP</t>
   </si>
   <si>
-    <t>Fecha y hora de generación: 26/11/2025 08:48:32</t>
+    <t>Fecha y hora de generación: 04/12/2025 08:46:46</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Corrcion ref a borrar
</commit_message>
<xml_diff>
--- a/VALORIZADO FALTANTES IMPO.xlsx
+++ b/VALORIZADO FALTANTES IMPO.xlsx
@@ -457,13 +457,13 @@
     <t>Valorizado</t>
   </si>
   <si>
-    <t>Período: 31/01/2026 07:43:42</t>
+    <t>Período: 31/01/2026 07:43:41</t>
   </si>
   <si>
     <t>COLGAAP</t>
   </si>
   <si>
-    <t>Fecha y hora de generación: 08/01/2026 07:44:15</t>
+    <t>Fecha y hora de generación: 09/01/2026 07:44:13</t>
   </si>
 </sst>
 </file>

</xml_diff>